<commit_message>
Inject David’s P-0722 jobs pack and shortened poster instructions.
Point volunteer PWA start_url at /retreat/ and keep retreat deploys shipping that manifest.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/jewelheart/jobs-v4.xlsx
+++ b/data/jewelheart/jobs-v4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\dev\RetreatVolunteer\Redesign\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\dev\RetreatVolunteer\Redesign\posters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C40E6AF-6727-4173-9355-094ADD505327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB4B331-2D40-420C-BEAE-8B7FE596078F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6970" yWindow="820" windowWidth="34980" windowHeight="16840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2970" yWindow="1320" windowWidth="34980" windowHeight="16840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jobs" sheetId="9" r:id="rId1"/>
@@ -41,12 +41,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="172">
   <si>
     <t>Job</t>
   </si>
   <si>
-    <t>Est
+    <t xml:space="preserve">Est
 Min</t>
   </si>
   <si>
@@ -62,40 +62,40 @@
     <t>Kitchen - end of day - full cleanup</t>
   </si>
   <si>
-    <t>Day 1
+    <t xml:space="preserve">Day 1
 Mon - Jul 20</t>
   </si>
   <si>
-    <t>Day 2
+    <t xml:space="preserve">Day 2
 Tue - July 21</t>
   </si>
   <si>
-    <t>Day 3
+    <t xml:space="preserve">Day 3
 Wed - Jul 22</t>
   </si>
   <si>
-    <t>Day 4
+    <t xml:space="preserve">Day 4
 Thu - July 23</t>
   </si>
   <si>
-    <t>Day 5
+    <t xml:space="preserve">Day 5
 Fri - Jul 24</t>
   </si>
   <si>
-    <t>Day 6
+    <t xml:space="preserve">Day 6
 Sat - Jul 25</t>
   </si>
   <si>
-    <t>Coffee &amp; snacks - evening brkdwn</t>
-  </si>
-  <si>
-    <t>Foyer &amp; lobby - vacuum</t>
+    <t>Coffee &amp;amp; snacks - evening brkdwn</t>
+  </si>
+  <si>
+    <t>Foyer &amp;amp; lobby - vacuum</t>
   </si>
   <si>
     <t>Front windows - clean</t>
   </si>
   <si>
-    <t>Coffee &amp; snacks - morning setup</t>
+    <t>Coffee &amp;amp; snacks - morning setup</t>
   </si>
   <si>
     <t>Men's room - clean, stock</t>
@@ -131,7 +131,7 @@
     <t>len</t>
   </si>
   <si>
-    <t>abbrev
+    <t xml:space="preserve">abbrev
  len</t>
   </si>
   <si>
@@ -192,7 +192,7 @@
     <t>e</t>
   </si>
   <si>
-    <t>Trash &amp; recycling - end of day</t>
+    <t>Trash &amp;amp; recycling - end of day</t>
   </si>
   <si>
     <t>Trash, recycle - end of day</t>
@@ -204,16 +204,16 @@
     <t>Twls, mop pds - laundr home</t>
   </si>
   <si>
-    <t>Unisx, lama bthrms, clean &amp; stock</t>
-  </si>
-  <si>
-    <t>Women's room, clean &amp; stock</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Urinals, check pads &amp; mop</t>
-  </si>
-  <si>
-    <t>Men's room, clean &amp; stock</t>
+    <t>Unisx, lama bthrms, clean &amp;amp; stock</t>
+  </si>
+  <si>
+    <t>Women's room, clean &amp;amp; stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Urinals, check pads &amp;amp; mop</t>
+  </si>
+  <si>
+    <t>Men's room, clean &amp;amp; stock</t>
   </si>
   <si>
     <t>XXXXX</t>
@@ -222,7 +222,7 @@
     <t>Front windows, clean</t>
   </si>
   <si>
-    <t>Foyer &amp; lobby, vacuum</t>
+    <t>Foyer &amp;amp; lobby, vacuum</t>
   </si>
   <si>
     <t>Coatrm, café hallwy, vacuum</t>
@@ -234,13 +234,13 @@
     <t>Tara Paradise, store, vacuum</t>
   </si>
   <si>
-    <t>Trash &amp; recycling</t>
+    <t>Trash &amp;amp; recycling</t>
   </si>
   <si>
     <t>Towels, mop pads, launder at home</t>
   </si>
   <si>
-    <t>Coffee &amp; snacks, evening brkdwn</t>
+    <t>Coffee &amp;amp; snacks, evening brkdwn</t>
   </si>
   <si>
     <t>Coffee, snacks, morning setup</t>
@@ -258,27 +258,27 @@
     <t>Café, lunch break, light cleanup</t>
   </si>
   <si>
-    <t>Day 6
+    <t xml:space="preserve">Day 6
 Sat, Jul 25</t>
   </si>
   <si>
-    <t>Day 5
+    <t xml:space="preserve">Day 5
 Fri, Jul 24</t>
   </si>
   <si>
-    <t>Day 4
+    <t xml:space="preserve">Day 4
 Thu, July 23</t>
   </si>
   <si>
-    <t>Day 3
+    <t xml:space="preserve">Day 3
 Wed, Jul 22</t>
   </si>
   <si>
-    <t>Day 2
+    <t xml:space="preserve">Day 2
 Tue, July 21</t>
   </si>
   <si>
-    <t>Day 1
+    <t xml:space="preserve">Day 1
 Mon, Jul 20</t>
   </si>
   <si>
@@ -309,9 +309,6 @@
     <t>djlewis@triadic.com</t>
   </si>
   <si>
-    <t>978-618-5709</t>
-  </si>
-  <si>
     <t>y</t>
   </si>
   <si>
@@ -324,26 +321,263 @@
     <t>Ann</t>
   </si>
   <si>
-    <t>Esckilsen</t>
-  </si>
-  <si>
     <t>kevinalexwoods@gmail.com</t>
   </si>
   <si>
-    <t>714-955-9394</t>
-  </si>
-  <si>
-    <t>612-453-9251</t>
-  </si>
-  <si>
     <t>arodgersreese63@gmail.com</t>
+  </si>
+  <si>
+    <t>✓ Kevin Woods</t>
+  </si>
+  <si>
+    <t>✓ Roland Driebergen</t>
+  </si>
+  <si>
+    <t>Roland Driebergen</t>
+  </si>
+  <si>
+    <t>✓ Sarah Hiser</t>
+  </si>
+  <si>
+    <t>✓ Figen Lacin</t>
+  </si>
+  <si>
+    <t>Susan Bradley</t>
+  </si>
+  <si>
+    <t>Diana Gonzalez</t>
+  </si>
+  <si>
+    <t>Sara Rutter</t>
+  </si>
+  <si>
+    <t>Ann Reese</t>
+  </si>
+  <si>
+    <t>Kevin Woods</t>
+  </si>
+  <si>
+    <t>David Lewis</t>
+  </si>
+  <si>
+    <t>Colleen Retherford</t>
+  </si>
+  <si>
+    <t>Sally Haines</t>
+  </si>
+  <si>
+    <t>Chris Frasz</t>
+  </si>
+  <si>
+    <t>Ronnie K</t>
+  </si>
+  <si>
+    <t>Sarah Hiser</t>
+  </si>
+  <si>
+    <t>Kayla Kern</t>
+  </si>
+  <si>
+    <t>✓ Peter Cha</t>
+  </si>
+  <si>
+    <t>✓ Heather Tasker</t>
+  </si>
+  <si>
+    <t>Heather Tasker</t>
+  </si>
+  <si>
+    <t>***Manual</t>
+  </si>
+  <si>
+    <t>***Entry</t>
+  </si>
+  <si>
+    <t>djlewis7865@yahoo.com</t>
+  </si>
+  <si>
+    <t>Andrew</t>
+  </si>
+  <si>
+    <t>Salisbury</t>
+  </si>
+  <si>
+    <t>drew.salis13@gmail.com</t>
+  </si>
+  <si>
+    <t>Reese</t>
+  </si>
+  <si>
+    <t>Chris</t>
+  </si>
+  <si>
+    <t>Frasz</t>
+  </si>
+  <si>
+    <t>cmfrasz@gmail.com</t>
+  </si>
+  <si>
+    <t>Colleen</t>
+  </si>
+  <si>
+    <t>Retherford</t>
+  </si>
+  <si>
+    <t>traveljones@hotmail.com</t>
+  </si>
+  <si>
+    <t>Diana</t>
+  </si>
+  <si>
+    <t>Gonzalez</t>
+  </si>
+  <si>
+    <t>kusan.diana@gmail.com</t>
+  </si>
+  <si>
+    <t>Figen</t>
+  </si>
+  <si>
+    <t>Lacin</t>
+  </si>
+  <si>
+    <t>figen.lacin@gmail.com</t>
+  </si>
+  <si>
+    <t>Hartmut</t>
+  </si>
+  <si>
+    <t>Sagolla</t>
+  </si>
+  <si>
+    <t>hartmut@jewelheart.org</t>
+  </si>
+  <si>
+    <t>Heather</t>
+  </si>
+  <si>
+    <t>MacKenzie</t>
+  </si>
+  <si>
+    <t>hmm715@gmail.com</t>
+  </si>
+  <si>
+    <t>Tasker</t>
+  </si>
+  <si>
+    <t>hltasker@yahoo.com</t>
+  </si>
+  <si>
+    <t>Kathy</t>
+  </si>
+  <si>
+    <t>Laritz</t>
+  </si>
+  <si>
+    <t>kathy@jewelheart.org</t>
+  </si>
+  <si>
+    <t>Kayla</t>
+  </si>
+  <si>
+    <t>Kern</t>
+  </si>
+  <si>
+    <t>kaylak1515@gmail.com</t>
+  </si>
+  <si>
+    <t>Peter</t>
+  </si>
+  <si>
+    <t>Cha</t>
+  </si>
+  <si>
+    <t>petercha92@gmail.com</t>
+  </si>
+  <si>
+    <t>Roland</t>
+  </si>
+  <si>
+    <t>Driebergen</t>
+  </si>
+  <si>
+    <t>r3bergen@gmail.com</t>
+  </si>
+  <si>
+    <t>Ronnie</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>bkoby4034@gmail.com</t>
+  </si>
+  <si>
+    <t>Sally</t>
+  </si>
+  <si>
+    <t>Haines</t>
+  </si>
+  <si>
+    <t>slawler@umich.edu</t>
+  </si>
+  <si>
+    <t>Sara</t>
+  </si>
+  <si>
+    <t>Rutter</t>
+  </si>
+  <si>
+    <t>srutterinhawaii@gmail.com</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Hiser</t>
+  </si>
+  <si>
+    <t>sarahhiser@gmail.com</t>
+  </si>
+  <si>
+    <t>Scott</t>
+  </si>
+  <si>
+    <t>Merwin</t>
+  </si>
+  <si>
+    <t>smerwin@umich.edu</t>
+  </si>
+  <si>
+    <t>734-576-2398</t>
+  </si>
+  <si>
+    <t>Seanna</t>
+  </si>
+  <si>
+    <t>Mueller-King</t>
+  </si>
+  <si>
+    <t>muellerking01@gmail.com</t>
+  </si>
+  <si>
+    <t>Susan</t>
+  </si>
+  <si>
+    <t>Bradley</t>
+  </si>
+  <si>
+    <t>bradleysf@gmail.com</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -428,8 +662,15 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -461,18 +702,48 @@
     <fill>
       <patternFill patternType="darkHorizontal">
         <fgColor rgb="FF808080"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="darkHorizontal">
-        <fgColor rgb="FF808080"/>
         <bgColor rgb="FFF8FFF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59996337778862885"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="darkHorizontal">
+        <fgColor rgb="FF808080"/>
+        <bgColor theme="5" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -529,10 +800,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -576,19 +848,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -601,7 +864,7 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -610,12 +873,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1637,20 +1922,21 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="22.36328125" style="2" customWidth="1"/>
-    <col min="2" max="7" width="24.6328125" style="3" customWidth="1"/>
+    <col min="2" max="7" width="32.6328125" style="3" customWidth="1"/>
     <col min="8" max="8" width="22.36328125" style="2" customWidth="1"/>
     <col min="9" max="9" width="5.90625" style="3" customWidth="1"/>
     <col min="10" max="10" width="6.1796875" style="2" customWidth="1"/>
-    <col min="11" max="11" width="22.36328125" style="15" customWidth="1"/>
-    <col min="12" max="13" width="8.7265625" style="2"/>
-    <col min="14" max="16384" width="8.7265625" style="3"/>
+    <col min="11" max="12" width="8.7265625" style="2"/>
+    <col min="13" max="13" width="8.7265625" style="3"/>
+    <col min="14" max="14" width="8.7265625" style="2"/>
+    <col min="15" max="16384" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="36">
+    <row r="1" spans="1:13" ht="36">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1678,359 +1964,362 @@
       <c r="I1" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="31">
-      <c r="A2" s="16" t="str">
+      <c r="M1" s="24"/>
+    </row>
+    <row r="2" spans="1:13" ht="53" customHeight="1">
+      <c r="A2" s="25" t="str">
         <f>Jobs!B2</f>
         <v>Café - lunch break - light cleanup</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="16" t="str">
-        <f>A2</f>
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+      <c r="H2" s="25" t="str">
+        <f t="shared" ref="H2:H18" si="0">A2</f>
         <v>Café - lunch break - light cleanup</v>
       </c>
       <c r="I2" s="1">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="31">
-      <c r="A3" s="16" t="str">
+      <c r="M2" s="26"/>
+    </row>
+    <row r="3" spans="1:13" ht="53" customHeight="1">
+      <c r="A3" s="25" t="str">
         <f>Jobs!B3</f>
         <v>Café - end of day - full cleanup</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="16" t="str">
-        <f>A3</f>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="H3" s="25" t="str">
+        <f t="shared" si="0"/>
         <v>Café - end of day - full cleanup</v>
       </c>
       <c r="I3" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="31">
-      <c r="A4" s="16" t="str">
+    <row r="4" spans="1:13" ht="53" customHeight="1">
+      <c r="A4" s="25" t="str">
         <f>Jobs!B4</f>
         <v>Kitchen - lunch break - light cleanup</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="16" t="str">
-        <f>A4</f>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4" s="25" t="str">
+        <f t="shared" si="0"/>
         <v>Kitchen - lunch break - light cleanup</v>
       </c>
       <c r="I4" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="31">
-      <c r="A5" s="16" t="str">
+    <row r="5" spans="1:13" ht="53" customHeight="1">
+      <c r="A5" s="25" t="str">
         <f>Jobs!B5</f>
         <v>Kitchen - end of day - full cleanup</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="16" t="str">
-        <f>A5</f>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5"/>
+      <c r="G5"/>
+      <c r="H5" s="25" t="str">
+        <f t="shared" si="0"/>
         <v>Kitchen - end of day - full cleanup</v>
       </c>
       <c r="I5" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="31">
-      <c r="A6" s="16" t="str">
+    <row r="6" spans="1:13" ht="53" customHeight="1">
+      <c r="A6" s="25" t="str">
         <f>Jobs!B6</f>
         <v>Coffee &amp; snacks - morning setup</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="16" t="str">
-        <f>A6</f>
+      <c r="B6"/>
+      <c r="C6"/>
+      <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6" s="25" t="str">
+        <f t="shared" si="0"/>
         <v>Coffee &amp; snacks - morning setup</v>
       </c>
       <c r="I6" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="31">
-      <c r="A7" s="16" t="str">
+    <row r="7" spans="1:13" ht="53" customHeight="1">
+      <c r="A7" s="25" t="str">
         <f>Jobs!B7</f>
         <v>Coffee &amp; snacks - evening brkdwn</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="16" t="str">
-        <f>A7</f>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="H7" s="25" t="str">
+        <f t="shared" si="0"/>
         <v>Coffee &amp; snacks - evening brkdwn</v>
       </c>
       <c r="I7" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="31">
-      <c r="A8" s="16" t="str">
+    <row r="8" spans="1:13" ht="53" customHeight="1">
+      <c r="A8" s="25" t="str">
         <f>Jobs!B8</f>
         <v>Dsh twls, mop pds - launder @home</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="17"/>
-      <c r="F8" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="17"/>
-      <c r="H8" s="16" t="str">
-        <f>A8</f>
+      <c r="B8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8"/>
+      <c r="F8" t="s">
+        <v>171</v>
+      </c>
+      <c r="G8"/>
+      <c r="H8" s="25" t="str">
+        <f t="shared" si="0"/>
         <v>Dsh twls, mop pds - launder @home</v>
       </c>
       <c r="I8" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="31">
-      <c r="A9" s="16" t="str">
+    <row r="9" spans="1:13" ht="53" customHeight="1">
+      <c r="A9" s="25" t="str">
         <f>Jobs!B9</f>
         <v>Trash &amp; recycling - end of day</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="16" t="str">
-        <f>A9</f>
+      <c r="B9"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9" s="25" t="str">
+        <f t="shared" si="0"/>
         <v>Trash &amp; recycling - end of day</v>
       </c>
       <c r="I9" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="31">
-      <c r="A10" s="16" t="str">
+    <row r="10" spans="1:13" ht="53" customHeight="1">
+      <c r="A10" s="27" t="str">
         <f>Jobs!B10</f>
         <v>Tara Paradise, store - vacuum</v>
       </c>
-      <c r="B10" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" s="17"/>
-      <c r="H10" s="16" t="str">
-        <f>A10</f>
+      <c r="B10" t="s">
+        <v>171</v>
+      </c>
+      <c r="C10"/>
+      <c r="D10" t="s">
+        <v>171</v>
+      </c>
+      <c r="E10"/>
+      <c r="F10" t="s">
+        <v>171</v>
+      </c>
+      <c r="G10"/>
+      <c r="H10" s="27" t="str">
+        <f t="shared" si="0"/>
         <v>Tara Paradise, store - vacuum</v>
       </c>
       <c r="I10" s="1">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="31">
-      <c r="A11" s="16" t="str">
+      <c r="M10" s="26"/>
+    </row>
+    <row r="11" spans="1:13" ht="53" customHeight="1">
+      <c r="A11" s="27" t="str">
         <f>Jobs!B11</f>
         <v>JH office, main hallway - vacuum</v>
       </c>
-      <c r="B11" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G11" s="17"/>
-      <c r="H11" s="16" t="str">
-        <f>A11</f>
+      <c r="B11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11" t="s">
+        <v>171</v>
+      </c>
+      <c r="E11"/>
+      <c r="F11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G11"/>
+      <c r="H11" s="27" t="str">
+        <f t="shared" si="0"/>
         <v>JH office, main hallway - vacuum</v>
       </c>
       <c r="I11" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="31">
-      <c r="A12" s="16" t="str">
+    <row r="12" spans="1:13" ht="53" customHeight="1">
+      <c r="A12" s="27" t="str">
         <f>Jobs!B12</f>
         <v>Coatrm, café hallway - vacuum</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="16" t="str">
-        <f>A12</f>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
+      <c r="H12" s="27" t="str">
+        <f t="shared" si="0"/>
         <v>Coatrm, café hallway - vacuum</v>
       </c>
       <c r="I12" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="31">
-      <c r="A13" s="16" t="str">
+    <row r="13" spans="1:13" ht="53" customHeight="1">
+      <c r="A13" s="27" t="str">
         <f>Jobs!B13</f>
         <v>Foyer &amp; lobby - vacuum</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="17"/>
-      <c r="E13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G13" s="17"/>
-      <c r="H13" s="16" t="str">
-        <f>A13</f>
+      <c r="B13" t="s">
+        <v>171</v>
+      </c>
+      <c r="C13" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13"/>
+      <c r="E13" t="s">
+        <v>171</v>
+      </c>
+      <c r="F13" t="s">
+        <v>171</v>
+      </c>
+      <c r="G13"/>
+      <c r="H13" s="27" t="str">
+        <f t="shared" si="0"/>
         <v>Foyer &amp; lobby - vacuum</v>
       </c>
       <c r="I13" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="31">
-      <c r="A14" s="16" t="str">
+    <row r="14" spans="1:13" ht="53" customHeight="1">
+      <c r="A14" s="27" t="str">
         <f>Jobs!B14</f>
         <v>Front windows - clean</v>
       </c>
-      <c r="B14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="17"/>
-      <c r="E14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G14" s="17"/>
-      <c r="H14" s="16" t="str">
-        <f>A14</f>
+      <c r="B14" t="s">
+        <v>171</v>
+      </c>
+      <c r="C14" t="s">
+        <v>171</v>
+      </c>
+      <c r="D14"/>
+      <c r="E14" t="s">
+        <v>171</v>
+      </c>
+      <c r="F14" t="s">
+        <v>171</v>
+      </c>
+      <c r="G14"/>
+      <c r="H14" s="27" t="str">
+        <f t="shared" si="0"/>
         <v>Front windows - clean</v>
       </c>
       <c r="I14" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="31">
-      <c r="A15" s="16" t="str">
+    <row r="15" spans="1:13" ht="53" customHeight="1">
+      <c r="A15" s="30" t="str">
         <f>Jobs!B15</f>
         <v>Men's room - clean, stock</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="16" t="str">
-        <f>A15</f>
+      <c r="B15"/>
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+      <c r="G15"/>
+      <c r="H15" s="30" t="str">
+        <f t="shared" si="0"/>
         <v>Men's room - clean, stock</v>
       </c>
       <c r="I15" s="1">
         <v>10</v>
       </c>
-      <c r="K15" s="18"/>
-    </row>
-    <row r="16" spans="1:11" ht="31">
-      <c r="A16" s="16" t="str">
+      <c r="M15" s="26"/>
+    </row>
+    <row r="16" spans="1:13" ht="53" customHeight="1">
+      <c r="A16" s="30" t="str">
         <f>Jobs!B16</f>
         <v xml:space="preserve"> Urinals - check pads, mop (x2)</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="16" t="str">
-        <f>A16</f>
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16"/>
+      <c r="H16" s="30" t="str">
+        <f t="shared" si="0"/>
         <v xml:space="preserve"> Urinals - check pads, mop (x2)</v>
       </c>
       <c r="I16" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="31">
-      <c r="A17" s="16" t="str">
+    <row r="17" spans="1:9" ht="53" customHeight="1">
+      <c r="A17" s="30" t="str">
         <f>Jobs!B17</f>
         <v>Women's room - clean, stock</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="16" t="str">
-        <f>A17</f>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="H17" s="30" t="str">
+        <f t="shared" si="0"/>
         <v>Women's room - clean, stock</v>
       </c>
       <c r="I17" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="31">
-      <c r="A18" s="16" t="str">
+    <row r="18" spans="1:9" ht="53" customHeight="1">
+      <c r="A18" s="30" t="str">
         <f>Jobs!B18</f>
         <v>Unisx, lama bathrms - clean, stock</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="16" t="str">
-        <f>A18</f>
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18" s="30" t="str">
+        <f t="shared" si="0"/>
         <v>Unisx, lama bathrms - clean, stock</v>
       </c>
       <c r="I18" s="1">
@@ -2039,7 +2328,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.1" footer="0.1"/>
-  <pageSetup fitToWidth="2" fitToHeight="2" orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="81" fitToWidth="2" fitToHeight="2" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2051,13 +2340,13 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="39.26953125" style="20" customWidth="1"/>
+    <col min="1" max="1" width="39.26953125" style="17" customWidth="1"/>
     <col min="2" max="7" width="24.6328125" style="3" customWidth="1"/>
     <col min="8" max="16384" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="36">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -2083,273 +2372,271 @@
       <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5"/>
+      <c r="G5"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
+      <c r="B6"/>
+      <c r="C6"/>
+      <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6"/>
+      <c r="G6"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="17"/>
+      <c r="B8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8"/>
+      <c r="F8" t="s">
+        <v>171</v>
+      </c>
+      <c r="G8"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="B9"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" s="17"/>
+      <c r="B10" t="s">
+        <v>171</v>
+      </c>
+      <c r="C10"/>
+      <c r="D10" t="s">
+        <v>171</v>
+      </c>
+      <c r="E10"/>
+      <c r="F10" t="s">
+        <v>171</v>
+      </c>
+      <c r="G10"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G11" s="17"/>
+      <c r="B11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11" t="s">
+        <v>171</v>
+      </c>
+      <c r="E11"/>
+      <c r="F11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G11"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="17"/>
-      <c r="E13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G13" s="17"/>
+      <c r="B13" t="s">
+        <v>171</v>
+      </c>
+      <c r="C13" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13"/>
+      <c r="E13" t="s">
+        <v>171</v>
+      </c>
+      <c r="F13" t="s">
+        <v>171</v>
+      </c>
+      <c r="G13"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
     </row>
     <row r="14" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="17"/>
-      <c r="E14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G14" s="17"/>
+      <c r="B14" t="s">
+        <v>171</v>
+      </c>
+      <c r="C14" t="s">
+        <v>171</v>
+      </c>
+      <c r="D14"/>
+      <c r="E14" t="s">
+        <v>171</v>
+      </c>
+      <c r="F14" t="s">
+        <v>171</v>
+      </c>
+      <c r="G14"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
+      <c r="B15"/>
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+      <c r="G15"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17"/>
       <c r="H17" s="3"/>
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" ht="16" customHeight="1">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
       <c r="H18" s="3"/>
     </row>
   </sheetData>
@@ -2360,223 +2647,371 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{692AD9D2-5874-44CD-9662-76B929B1C53D}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.26953125" style="26" customWidth="1"/>
-    <col min="2" max="2" width="16.453125" style="26" customWidth="1"/>
-    <col min="3" max="3" width="34.36328125" style="26" customWidth="1"/>
-    <col min="4" max="4" width="29.54296875" style="26" customWidth="1"/>
-    <col min="5" max="6" width="8.7265625" style="26"/>
+    <col min="1" max="1" width="12.26953125" style="23" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" style="23" customWidth="1"/>
+    <col min="3" max="3" width="34.36328125" style="23" customWidth="1"/>
+    <col min="4" max="4" width="29.54296875" style="23" customWidth="1"/>
+    <col min="5" max="6" width="8.7265625" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="23" customFormat="1">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:6" s="20" customFormat="1">
+      <c r="A1" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="21" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B7" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C7" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D7" s="22"/>
+      <c r="E7" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="F7" s="22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="F2" s="25" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="25" t="s">
+      <c r="B15" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="25" t="s">
+      <c r="C15" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="25"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="25"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="25"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="25"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="25"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="25"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="25"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
+      <c r="A16" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="25"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
+      <c r="A17" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="25"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
+      <c r="A18" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="25"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
+      <c r="A19" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="25"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
+      <c r="A20" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>